<commit_message>
Translate Excel finished (key access still personal)
</commit_message>
<xml_diff>
--- a/pythonWork/pythonSource/tools/LANGTRANSL/tests/testexcel.xlsx
+++ b/pythonWork/pythonSource/tools/LANGTRANSL/tests/testexcel.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Master Entity</t>
+          <t>Main entity</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -474,7 +474,6 @@
           <t>Hauptentität  Entity-Name</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -502,7 +501,6 @@
           <t>Hauptentität  Entity-Name</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -520,7 +518,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>Master entity with 3 children with attributes and classifications
-Displayed on all zoom levels (0-4)
+Displayed at all zoom levels (0-4)
 single attribute Unique key</t>
         </is>
       </c>
@@ -536,7 +534,6 @@
           <t>Hauptentität  Entity--Description</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -544,15 +541,11 @@
           <t>ENTI119-tooltip</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Hauptentität  Entity--Tooltip</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -567,7 +560,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Main Entity</t>
+          <t>Father entity</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -580,7 +573,6 @@
           <t>Hauptentität-&gt;Vaterentität  - Synonym-1</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -600,7 +592,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1. exemple: Entité maître</t>
+          <t>1. Exemple d'entité maître</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -608,7 +600,6 @@
           <t>Hauptentität  - Example-1</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -623,7 +614,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2. Example: Master Entity</t>
+          <t>2. Master entity example.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -636,7 +627,6 @@
           <t>Hauptentität  - Example-2</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -656,7 +646,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1. Example: Attribut</t>
+          <t>1. Exemple d'attributs</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -664,7 +654,6 @@
           <t>erste Erscheinung  - Example-1</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -692,7 +681,6 @@
           <t>Hauptentität-&gt;Name  Attribute-Name</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -712,7 +700,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Attribut descriptif, obligatoire avec domaine, affiché au niveau de zoom 0-2</t>
+          <t>Attribut descriptif obligatoire avec plage, affiché au niveau de zoom 0-2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -720,7 +708,6 @@
           <t>Hauptentität-&gt;Name  Attribute-Description</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -728,15 +715,11 @@
           <t>ATTR123-tooltip</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Hauptentität-&gt;Name  Attribute-Tooltip</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -764,7 +747,6 @@
           <t>XMLTYPE  Domain-Name</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -772,15 +754,11 @@
           <t>DOMA90-descr</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>XMLTYPE  Domain-Description</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -800,7 +778,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>email Address</t>
+          <t>adresse électronique</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -808,7 +786,6 @@
           <t>email Address  Domain-Name</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -836,7 +813,6 @@
           <t>email Address  Domain-Description</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -844,15 +820,11 @@
           <t>RELA138-fromto</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Relation -Kind Entität1 =&gt; Hauptentität</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -860,15 +832,11 @@
           <t>RELA138-tofrom</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>Relation -Hauptentität =&gt; Kind Entität1</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -896,7 +864,6 @@
           <t>Relation -Zusätzliche Einheit =&gt; Rollen-Entität 2</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -924,7 +891,6 @@
           <t>Relation -Rollen-Entität 2 =&gt; Zusätzliche Einheit</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">

</xml_diff>